<commit_message>
test: improve aggregate conformance fixtures with comprehensive edge cases
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/aggregate/basic_aggregates.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/aggregate/basic_aggregates.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="MixedData" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,39 +21,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">amt</t>
   </si>
   <si>
+    <t xml:space="preserve">sum_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">average_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">median_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product_literal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">double</t>
+  </si>
+  <si>
     <t xml:space="preserve">mixed</t>
   </si>
   <si>
-    <t xml:space="preserve">sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">count</t>
-  </si>
-  <si>
     <t xml:space="preserve">counta</t>
   </si>
   <si>
     <t xml:space="preserve">countblank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">average</t>
-  </si>
-  <si>
-    <t xml:space="preserve">min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">median</t>
-  </si>
-  <si>
-    <t xml:space="preserve">product</t>
   </si>
   <si>
     <t xml:space="preserve">text</t>
@@ -134,11 +138,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+  <cellXfs count="1">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -335,7 +335,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -366,52 +366,42 @@
       <c r="I1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="0" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
         <v>1000</v>
       </c>
+      <c r="B2" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
       <c r="C2" s="0" t="n">
-        <f aca="false">SUM(A:A)</f>
-        <v>24600</v>
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
       </c>
       <c r="D2" s="0" t="n">
-        <f aca="false">COUNT(A:A)</f>
-        <v>10</v>
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
       </c>
       <c r="E2" s="0" t="n">
-        <f aca="false">COUNTA(B:B)</f>
-        <v>7</v>
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
       </c>
       <c r="F2" s="0" t="n">
-        <f aca="false">COUNTBLANK(B:B)</f>
-        <v>1048569</v>
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
       </c>
       <c r="G2" s="0" t="n">
-        <f aca="false">AVERAGE(A:A)</f>
-        <v>2460</v>
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
       </c>
       <c r="H2" s="0" t="n">
-        <f aca="false">MIN(A:A)</f>
-        <v>0</v>
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
       </c>
       <c r="I2" s="0" t="n">
-        <f aca="false">MAX(A:A)</f>
-        <v>7500</v>
-      </c>
-      <c r="J2" s="0" t="n">
-        <f aca="false">MEDIAN(A:A)</f>
-        <v>1850</v>
-      </c>
-      <c r="K2" s="0" t="n">
-        <f aca="false">PRODUCT(2,3,4)</f>
-        <v>24</v>
+        <f aca="false">A2*2</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -419,29 +409,147 @@
         <v>2500</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>42</v>
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I3" s="0" t="n">
+        <f aca="false">A3*2</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>11</v>
+      <c r="B4" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I4" s="0" t="n">
+        <f aca="false">A4*2</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="n">
         <v>5000</v>
       </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I5" s="0" t="n">
+        <f aca="false">A5*2</f>
+        <v>10000</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="n">
-        <v>150</v>
-      </c>
-      <c r="B6" s="1" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+        <v>-150</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I6" s="0" t="n">
+        <f aca="false">A6*2</f>
+        <v>-300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -449,20 +557,110 @@
         <v>3000</v>
       </c>
       <c r="B7" s="0" t="n">
-        <v>0</v>
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I7" s="0" t="n">
+        <f aca="false">A7*2</f>
+        <v>6000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="n">
         <v>7500</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <f aca="false">A8*2</f>
+        <v>15000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="B9" s="0" t="s">
-        <v>12</v>
+      <c r="B9" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I9" s="0" t="n">
+        <f aca="false">A9*2</f>
+        <v>500</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -470,12 +668,198 @@
         <v>4000</v>
       </c>
       <c r="B10" s="0" t="n">
-        <v>100</v>
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H10" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <f aca="false">A10*2</f>
+        <v>8000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="n">
         <v>1200</v>
+      </c>
+      <c r="B11" s="0" t="n">
+        <f aca="false">SUM(A:A)</f>
+        <v>24300</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <f aca="false">COUNT(A:A)</f>
+        <v>10</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <f aca="false">AVERAGE(A:A)</f>
+        <v>2430</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <f aca="false">MIN(A:A)</f>
+        <v>-150</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <f aca="false">MAX(A:A)</f>
+        <v>7500</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <f aca="false">MEDIAN(A:A)</f>
+        <v>1850</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <f aca="false">PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <f aca="false">A11*2</f>
+        <v>2400</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>100</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="0" t="n">
+        <f aca="false">COUNTA(A:A)</f>
+        <v>6</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <f aca="false">COUNTBLANK(A:A)</f>
+        <v>1048570</v>
       </c>
     </row>
   </sheetData>

</xml_diff>